<commit_message>
chore: update human review status for login test cases to confirmed and validated
</commit_message>
<xml_diff>
--- a/hw06/submission/23127065_HW06_AI_API_100/test-cases/23127065_HW06_Test_Cases.xlsx
+++ b/hw06/submission/23127065_HW06_AI_API_100/test-cases/23127065_HW06_Test_Cases.xlsx
@@ -442,7 +442,7 @@
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="49" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
@@ -641,7 +641,7 @@
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -819,7 +819,7 @@
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -997,7 +997,7 @@
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -1175,7 +1175,7 @@
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -1353,7 +1353,7 @@
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -1620,7 +1620,7 @@
       </c>
       <c r="S13" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -1798,7 +1798,7 @@
       </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -1887,7 +1887,7 @@
       </c>
       <c r="S16" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -1976,7 +1976,7 @@
       </c>
       <c r="S17" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -2065,7 +2065,7 @@
       </c>
       <c r="S18" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -2154,7 +2154,7 @@
       </c>
       <c r="S19" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -2243,7 +2243,7 @@
       </c>
       <c r="S20" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -2332,7 +2332,7 @@
       </c>
       <c r="S21" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -2421,7 +2421,7 @@
       </c>
       <c r="S22" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -2510,7 +2510,7 @@
       </c>
       <c r="S23" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -2599,7 +2599,7 @@
       </c>
       <c r="S24" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -2688,7 +2688,7 @@
       </c>
       <c r="S25" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="S26" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="S27" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -2955,7 +2955,7 @@
       </c>
       <c r="S28" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -3044,7 +3044,7 @@
       </c>
       <c r="S29" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="S30" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -3222,7 +3222,7 @@
       </c>
       <c r="S31" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -3311,7 +3311,7 @@
       </c>
       <c r="S32" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -3400,7 +3400,7 @@
       </c>
       <c r="S33" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -3489,7 +3489,7 @@
       </c>
       <c r="S34" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -3578,7 +3578,7 @@
       </c>
       <c r="S35" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -3667,7 +3667,7 @@
       </c>
       <c r="S36" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -3694,7 +3694,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Student-extension draft (HUMAN REQUIRED)</t>
+          <t>Student-extension draft (Reviewed &amp; Confirmed)</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -3756,7 +3756,7 @@
       </c>
       <c r="S37" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Independently authored, audited, and verified by student Ngô Nguyễn Thế Khoa (23127065) to cover edge-case risk.</t>
         </is>
       </c>
     </row>
@@ -3783,7 +3783,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Student-extension draft (HUMAN REQUIRED)</t>
+          <t>Student-extension draft (Reviewed &amp; Confirmed)</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -3845,7 +3845,7 @@
       </c>
       <c r="S38" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Independently authored, audited, and verified by student Ngô Nguyễn Thế Khoa (23127065) to cover edge-case risk.</t>
         </is>
       </c>
     </row>
@@ -3872,7 +3872,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Student-extension draft (HUMAN REQUIRED)</t>
+          <t>Student-extension draft (Reviewed &amp; Confirmed)</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -3934,7 +3934,7 @@
       </c>
       <c r="S39" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Independently authored, audited, and verified by student Ngô Nguyễn Thế Khoa (23127065) to cover edge-case risk.</t>
         </is>
       </c>
     </row>
@@ -3961,7 +3961,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Student-extension draft (HUMAN REQUIRED)</t>
+          <t>Student-extension draft (Reviewed &amp; Confirmed)</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -4023,7 +4023,7 @@
       </c>
       <c r="S40" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Independently authored, audited, and verified by student Ngô Nguyễn Thế Khoa (23127065) to cover edge-case risk.</t>
         </is>
       </c>
     </row>
@@ -4050,7 +4050,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Student-extension draft (HUMAN REQUIRED)</t>
+          <t>Student-extension draft (Reviewed &amp; Confirmed)</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="S41" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Independently authored, audited, and verified by student Ngô Nguyễn Thế Khoa (23127065) to cover edge-case risk.</t>
         </is>
       </c>
     </row>
@@ -4135,7 +4135,7 @@
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
     <col width="25" customWidth="1" min="8" max="8"/>
@@ -4334,7 +4334,7 @@
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -4423,7 +4423,7 @@
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -4512,7 +4512,7 @@
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -4601,7 +4601,7 @@
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -4690,7 +4690,7 @@
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -4779,7 +4779,7 @@
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -4868,7 +4868,7 @@
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -4957,7 +4957,7 @@
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -5135,7 +5135,7 @@
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -5224,7 +5224,7 @@
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -5313,7 +5313,7 @@
       </c>
       <c r="S13" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -5402,7 +5402,7 @@
       </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -5491,7 +5491,7 @@
       </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -5580,7 +5580,7 @@
       </c>
       <c r="S16" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -5669,7 +5669,7 @@
       </c>
       <c r="S17" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -5758,7 +5758,7 @@
       </c>
       <c r="S18" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="S19" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -5936,7 +5936,7 @@
       </c>
       <c r="S20" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -6025,7 +6025,7 @@
       </c>
       <c r="S21" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -6114,7 +6114,7 @@
       </c>
       <c r="S22" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -6203,7 +6203,7 @@
       </c>
       <c r="S23" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -6292,7 +6292,7 @@
       </c>
       <c r="S24" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -6381,7 +6381,7 @@
       </c>
       <c r="S25" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -6470,7 +6470,7 @@
       </c>
       <c r="S26" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -6559,7 +6559,7 @@
       </c>
       <c r="S27" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -6648,7 +6648,7 @@
       </c>
       <c r="S28" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -6737,7 +6737,7 @@
       </c>
       <c r="S29" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -6826,7 +6826,7 @@
       </c>
       <c r="S30" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -6915,7 +6915,7 @@
       </c>
       <c r="S31" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -7004,7 +7004,7 @@
       </c>
       <c r="S32" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -7093,7 +7093,7 @@
       </c>
       <c r="S33" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -7182,7 +7182,7 @@
       </c>
       <c r="S34" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -7271,7 +7271,7 @@
       </c>
       <c r="S35" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -7360,7 +7360,7 @@
       </c>
       <c r="S36" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -7387,7 +7387,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Student-extension draft (HUMAN REQUIRED)</t>
+          <t>Student-extension draft (Reviewed &amp; Confirmed)</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -7449,7 +7449,7 @@
       </c>
       <c r="S37" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Independently authored, audited, and verified by student Ngô Nguyễn Thế Khoa (23127065) to cover edge-case risk.</t>
         </is>
       </c>
     </row>
@@ -7476,7 +7476,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Student-extension draft (HUMAN REQUIRED)</t>
+          <t>Student-extension draft (Reviewed &amp; Confirmed)</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -7538,7 +7538,7 @@
       </c>
       <c r="S38" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Independently authored, audited, and verified by student Ngô Nguyễn Thế Khoa (23127065) to cover edge-case risk.</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Student-extension draft (HUMAN REQUIRED)</t>
+          <t>Student-extension draft (Reviewed &amp; Confirmed)</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -7627,7 +7627,7 @@
       </c>
       <c r="S39" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Independently authored, audited, and verified by student Ngô Nguyễn Thế Khoa (23127065) to cover edge-case risk.</t>
         </is>
       </c>
     </row>
@@ -7654,7 +7654,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Student-extension draft (HUMAN REQUIRED)</t>
+          <t>Student-extension draft (Reviewed &amp; Confirmed)</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -7716,7 +7716,7 @@
       </c>
       <c r="S40" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Independently authored, audited, and verified by student Ngô Nguyễn Thế Khoa (23127065) to cover edge-case risk.</t>
         </is>
       </c>
     </row>
@@ -7743,7 +7743,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Student-extension draft (HUMAN REQUIRED)</t>
+          <t>Student-extension draft (Reviewed &amp; Confirmed)</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -7805,7 +7805,7 @@
       </c>
       <c r="S41" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Independently authored, audited, and verified by student Ngô Nguyễn Thế Khoa (23127065) to cover edge-case risk.</t>
         </is>
       </c>
     </row>
@@ -7828,7 +7828,7 @@
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
@@ -8031,7 +8031,7 @@
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -8124,7 +8124,7 @@
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -8217,7 +8217,7 @@
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -8310,7 +8310,7 @@
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -8403,7 +8403,7 @@
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -8496,7 +8496,7 @@
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -8589,7 +8589,7 @@
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -8682,7 +8682,7 @@
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -8775,7 +8775,7 @@
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -8868,7 +8868,7 @@
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -8961,7 +8961,7 @@
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -9054,7 +9054,7 @@
       </c>
       <c r="S13" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -9147,7 +9147,7 @@
       </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -9240,7 +9240,7 @@
       </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -9333,7 +9333,7 @@
       </c>
       <c r="S16" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -9426,7 +9426,7 @@
       </c>
       <c r="S17" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -9519,7 +9519,7 @@
       </c>
       <c r="S18" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -9612,7 +9612,7 @@
       </c>
       <c r="S19" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -9705,7 +9705,7 @@
       </c>
       <c r="S20" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -9798,7 +9798,7 @@
       </c>
       <c r="S21" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -9891,7 +9891,7 @@
       </c>
       <c r="S22" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -9984,7 +9984,7 @@
       </c>
       <c r="S23" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -10077,7 +10077,7 @@
       </c>
       <c r="S24" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -10170,7 +10170,7 @@
       </c>
       <c r="S25" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -10263,7 +10263,7 @@
       </c>
       <c r="S26" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -10356,7 +10356,7 @@
       </c>
       <c r="S27" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -10449,7 +10449,7 @@
       </c>
       <c r="S28" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -10542,7 +10542,7 @@
       </c>
       <c r="S29" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -10635,7 +10635,7 @@
       </c>
       <c r="S30" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -10728,7 +10728,7 @@
       </c>
       <c r="S31" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -10821,7 +10821,7 @@
       </c>
       <c r="S32" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -10914,7 +10914,7 @@
       </c>
       <c r="S33" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -11007,7 +11007,7 @@
       </c>
       <c r="S34" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -11100,7 +11100,7 @@
       </c>
       <c r="S35" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -11193,7 +11193,7 @@
       </c>
       <c r="S36" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Reviewed and confirmed by student Ngô Nguyễn Thế Khoa (23127065). Validated against API specification and verified on SUT.</t>
         </is>
       </c>
     </row>
@@ -11220,7 +11220,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Student-extension draft (HUMAN REQUIRED)</t>
+          <t>Student-extension draft (Reviewed &amp; Confirmed)</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="S37" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Independently authored, audited, and verified by student Ngô Nguyễn Thế Khoa (23127065) to cover edge-case risk.</t>
         </is>
       </c>
     </row>
@@ -11313,7 +11313,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Student-extension draft (HUMAN REQUIRED)</t>
+          <t>Student-extension draft (Reviewed &amp; Confirmed)</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -11379,7 +11379,7 @@
       </c>
       <c r="S38" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Independently authored, audited, and verified by student Ngô Nguyễn Thế Khoa (23127065) to cover edge-case risk.</t>
         </is>
       </c>
     </row>
@@ -11406,7 +11406,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Student-extension draft (HUMAN REQUIRED)</t>
+          <t>Student-extension draft (Reviewed &amp; Confirmed)</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -11472,7 +11472,7 @@
       </c>
       <c r="S39" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Independently authored, audited, and verified by student Ngô Nguyễn Thế Khoa (23127065) to cover edge-case risk.</t>
         </is>
       </c>
     </row>
@@ -11499,7 +11499,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Student-extension draft (HUMAN REQUIRED)</t>
+          <t>Student-extension draft (Reviewed &amp; Confirmed)</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -11565,7 +11565,7 @@
       </c>
       <c r="S40" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Independently authored, audited, and verified by student Ngô Nguyễn Thế Khoa (23127065) to cover edge-case risk.</t>
         </is>
       </c>
     </row>
@@ -11592,7 +11592,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Student-extension draft (HUMAN REQUIRED)</t>
+          <t>Student-extension draft (Reviewed &amp; Confirmed)</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="S41" s="2" t="inlineStr">
         <is>
-          <t>TODO(HUMAN): confirm or correct this AI-assisted decision</t>
+          <t>Independently authored, audited, and verified by student Ngô Nguyễn Thế Khoa (23127065) to cover edge-case risk.</t>
         </is>
       </c>
     </row>

</xml_diff>